<commit_message>
day 5 and day6
</commit_message>
<xml_diff>
--- a/leetcode qsn.xlsx
+++ b/leetcode qsn.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AEB1550-F22F-4F70-9F2E-5E32F56C0503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74E93F4-7A52-4B77-BAF0-9649BAFFA95C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARRAYS" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,8 @@
     <sheet name="GREEDY, DFS" sheetId="5" r:id="rId5"/>
     <sheet name="TREE, BFS" sheetId="6" r:id="rId6"/>
     <sheet name="BINARY SEARCH, HEAPS" sheetId="7" r:id="rId7"/>
-    <sheet name="BACKTRACKING, STACK" sheetId="8" r:id="rId8"/>
-    <sheet name="LINKED LIST" sheetId="9" r:id="rId9"/>
+    <sheet name="LINKED LIST" sheetId="9" r:id="rId8"/>
+    <sheet name="BACKTRACKING, STACK" sheetId="8" r:id="rId9"/>
     <sheet name="SLIDING WINDOW" sheetId="10" r:id="rId10"/>
     <sheet name="DESIGN, GRAPH" sheetId="11" r:id="rId11"/>
     <sheet name="TRIE, SEGMENT TREE" sheetId="12" r:id="rId12"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="361">
   <si>
     <t>Arrays Easy</t>
   </si>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B4" s="6"/>
       <c r="F4" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>233</v>
@@ -3974,7 +3974,9 @@
         <v>240</v>
       </c>
       <c r="B9" s="6"/>
-      <c r="F9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>358</v>
+      </c>
       <c r="G9" s="8" t="s">
         <v>241</v>
       </c>
@@ -4014,7 +4016,7 @@
       </c>
       <c r="B13" s="6"/>
       <c r="F13" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>248</v>
@@ -4506,159 +4508,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="K2" s="4"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="K4" s="4"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="3" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>281</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="K7" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="F14" s="8" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="F15" s="8" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="F16" s="8" t="s">
-        <v>295</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
-    <hyperlink ref="F2" r:id="rId2" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
-    <hyperlink ref="F3" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
-    <hyperlink ref="A4" r:id="rId5" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
-    <hyperlink ref="F4" r:id="rId6" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
-    <hyperlink ref="A5" r:id="rId7" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
-    <hyperlink ref="F5" r:id="rId8" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
-    <hyperlink ref="A6" r:id="rId9" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
-    <hyperlink ref="F6" r:id="rId10" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
-    <hyperlink ref="A7" r:id="rId11" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
-    <hyperlink ref="F7" r:id="rId12" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
-    <hyperlink ref="A10" r:id="rId13" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
-    <hyperlink ref="F10" r:id="rId14" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
-    <hyperlink ref="A11" r:id="rId15" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
-    <hyperlink ref="F11" r:id="rId16" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
-    <hyperlink ref="A12" r:id="rId17" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
-    <hyperlink ref="F12" r:id="rId18" xr:uid="{00000000-0004-0000-0700-000011000000}"/>
-    <hyperlink ref="A13" r:id="rId19" xr:uid="{00000000-0004-0000-0700-000012000000}"/>
-    <hyperlink ref="F13" r:id="rId20" xr:uid="{00000000-0004-0000-0700-000013000000}"/>
-    <hyperlink ref="F14" r:id="rId21" xr:uid="{00000000-0004-0000-0700-000014000000}"/>
-    <hyperlink ref="F15" r:id="rId22" xr:uid="{00000000-0004-0000-0700-000015000000}"/>
-    <hyperlink ref="F16" r:id="rId23" xr:uid="{00000000-0004-0000-0700-000016000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4819,4 +4668,157 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="K7" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F14" s="8" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F15" s="8" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F16" s="8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="F2" r:id="rId2" xr:uid="{00000000-0004-0000-0700-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{00000000-0004-0000-0700-000002000000}"/>
+    <hyperlink ref="F3" r:id="rId4" xr:uid="{00000000-0004-0000-0700-000003000000}"/>
+    <hyperlink ref="A4" r:id="rId5" xr:uid="{00000000-0004-0000-0700-000004000000}"/>
+    <hyperlink ref="F4" r:id="rId6" xr:uid="{00000000-0004-0000-0700-000005000000}"/>
+    <hyperlink ref="A5" r:id="rId7" xr:uid="{00000000-0004-0000-0700-000006000000}"/>
+    <hyperlink ref="F5" r:id="rId8" xr:uid="{00000000-0004-0000-0700-000007000000}"/>
+    <hyperlink ref="A6" r:id="rId9" xr:uid="{00000000-0004-0000-0700-000008000000}"/>
+    <hyperlink ref="F6" r:id="rId10" xr:uid="{00000000-0004-0000-0700-000009000000}"/>
+    <hyperlink ref="A7" r:id="rId11" xr:uid="{00000000-0004-0000-0700-00000A000000}"/>
+    <hyperlink ref="F7" r:id="rId12" xr:uid="{00000000-0004-0000-0700-00000B000000}"/>
+    <hyperlink ref="A10" r:id="rId13" xr:uid="{00000000-0004-0000-0700-00000C000000}"/>
+    <hyperlink ref="F10" r:id="rId14" xr:uid="{00000000-0004-0000-0700-00000D000000}"/>
+    <hyperlink ref="A11" r:id="rId15" xr:uid="{00000000-0004-0000-0700-00000E000000}"/>
+    <hyperlink ref="F11" r:id="rId16" xr:uid="{00000000-0004-0000-0700-00000F000000}"/>
+    <hyperlink ref="A12" r:id="rId17" xr:uid="{00000000-0004-0000-0700-000010000000}"/>
+    <hyperlink ref="F12" r:id="rId18" xr:uid="{00000000-0004-0000-0700-000011000000}"/>
+    <hyperlink ref="A13" r:id="rId19" xr:uid="{00000000-0004-0000-0700-000012000000}"/>
+    <hyperlink ref="F13" r:id="rId20" xr:uid="{00000000-0004-0000-0700-000013000000}"/>
+    <hyperlink ref="F14" r:id="rId21" xr:uid="{00000000-0004-0000-0700-000014000000}"/>
+    <hyperlink ref="F15" r:id="rId22" xr:uid="{00000000-0004-0000-0700-000015000000}"/>
+    <hyperlink ref="F16" r:id="rId23" xr:uid="{00000000-0004-0000-0700-000016000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>